<commit_message>
21th commit: Updated unittest plan for InvestmentAccount class. Added unittesting for InvestmentAccount.
</commit_message>
<xml_diff>
--- a/tests/A02_pixell_test_plan_investment_account.xlsx
+++ b/tests/A02_pixell_test_plan_investment_account.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="36">
   <si>
     <t>#VALUE!</t>
   </si>
@@ -25,6 +25,9 @@
     <t>Developer:</t>
   </si>
   <si>
+    <t>Sven Beitenger</t>
+  </si>
+  <si>
     <t>Class Name:</t>
   </si>
   <si>
@@ -55,28 +58,72 @@
     <t>Attributes are set to parameter values.</t>
   </si>
   <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>account_number = 1172010
+client_number = 98765
+balance = 80000.85 created_date = date(2025,9,30), managment_fee = 3</t>
+  </si>
+  <si>
+    <t>All attributes are set.</t>
+  </si>
+  <si>
     <t>management fee has invalid type.</t>
   </si>
   <si>
+    <t>account_number = 1172010
+client_number = 98765
+balance = 80000.85 created_date = date(2025,9,30), managment_fee = "str"</t>
+  </si>
+  <si>
+    <t>managment_fee = 2.55</t>
+  </si>
+  <si>
     <t>get_service_charges</t>
   </si>
   <si>
     <t>date created more than 10 years ago</t>
   </si>
   <si>
+    <t>InvestmentAccount(1172010, 98765, 80000.85, date(2000,9,30), 3</t>
+  </si>
+  <si>
+    <t>service_charge = 0.50</t>
+  </si>
+  <si>
     <t>date created exactly 10 years ago.</t>
   </si>
   <si>
+    <t>InvestmentAccount(1172010, 98765, 80000.85, date(2015,10,1), 3</t>
+  </si>
+  <si>
     <t>date created within last 10 years.</t>
   </si>
   <si>
+    <t>InvestmentAccount(1172010, 98765, 80000.85, date(2020,10,1), 3</t>
+  </si>
+  <si>
+    <t>service_charge = 3.5</t>
+  </si>
+  <si>
     <t>__str__</t>
   </si>
   <si>
     <t>displays waived management fee when date created more than 10 years ago.</t>
   </si>
   <si>
+    <t>managment fee = "waived"</t>
+  </si>
+  <si>
     <t>displays  management fee when date created within last 10 years.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">InvestmentAccount(1172010, 98765, 80000.85, date(2020,10,1), 3
+</t>
+  </si>
+  <si>
+    <t>managment fee = 3</t>
   </si>
   <si>
     <t>Add more rows as necessary</t>
@@ -860,7 +907,9 @@
       <c r="B3" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="8"/>
+      <c r="C3" s="8" t="s">
+        <v>3</v>
+      </c>
       <c r="D3" s="9"/>
       <c r="E3" s="3"/>
       <c r="F3" s="3"/>
@@ -869,10 +918,10 @@
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
       <c r="A4" s="1"/>
       <c r="B4" s="10" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D4" s="12"/>
       <c r="E4" s="3"/>
@@ -891,128 +940,170 @@
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
       <c r="A6" s="1"/>
       <c r="B6" s="14" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C6" s="15" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D6" s="15" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E6" s="15" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F6" s="15" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G6" s="15" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5" customFormat="1" s="16">
+        <v>11</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="90" customFormat="1" s="16">
       <c r="A7" s="17"/>
       <c r="B7" s="18">
         <v>1</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D7" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="E7" s="20"/>
-      <c r="F7" s="20"/>
-      <c r="G7" s="20"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5" customFormat="1" s="16">
+        <v>13</v>
+      </c>
+      <c r="E7" s="20" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" s="20" t="s">
+        <v>15</v>
+      </c>
+      <c r="G7" s="20" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="88.5" customFormat="1" s="16">
       <c r="A8" s="17"/>
       <c r="B8" s="21">
         <v>2</v>
       </c>
       <c r="C8" s="22" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D8" s="22" t="s">
-        <v>13</v>
-      </c>
-      <c r="E8" s="20"/>
-      <c r="F8" s="20"/>
-      <c r="G8" s="23"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5" customFormat="1" s="16">
+        <v>17</v>
+      </c>
+      <c r="E8" s="20" t="s">
+        <v>14</v>
+      </c>
+      <c r="F8" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="G8" s="23" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="98.25" customFormat="1" s="16">
       <c r="A9" s="17"/>
       <c r="B9" s="18">
         <v>3</v>
       </c>
       <c r="C9" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" s="22" t="s">
+        <v>21</v>
+      </c>
+      <c r="E9" s="20" t="s">
+        <v>22</v>
+      </c>
+      <c r="F9" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="D9" s="22" t="s">
-        <v>15</v>
-      </c>
-      <c r="E9" s="20"/>
-      <c r="F9" s="23"/>
-      <c r="G9" s="23"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="19.5" customFormat="1" s="16">
+      <c r="G9" s="23" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="77.25" customFormat="1" s="16">
       <c r="A10" s="17"/>
       <c r="B10" s="18">
         <v>4</v>
       </c>
       <c r="C10" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="D10" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="E10" s="23" t="s">
+        <v>25</v>
+      </c>
+      <c r="F10" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="D10" s="22" t="s">
-        <v>16</v>
-      </c>
-      <c r="E10" s="23"/>
-      <c r="F10" s="23"/>
-      <c r="G10" s="23"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="19.5" customFormat="1" s="16">
+      <c r="G10" s="23" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="63" customFormat="1" s="16">
       <c r="A11" s="17"/>
       <c r="B11" s="18">
         <v>5</v>
       </c>
       <c r="C11" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="D11" s="22" t="s">
+        <v>26</v>
+      </c>
+      <c r="E11" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="F11" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="D11" s="22" t="s">
-        <v>17</v>
-      </c>
-      <c r="E11" s="20"/>
-      <c r="F11" s="23"/>
-      <c r="G11" s="23"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="44.25" customFormat="1" s="16">
+      <c r="G11" s="23" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="57.75" customFormat="1" s="16">
       <c r="A12" s="17"/>
       <c r="B12" s="21">
         <v>6</v>
       </c>
       <c r="C12" s="22" t="s">
-        <v>18</v>
+        <v>29</v>
       </c>
       <c r="D12" s="22" t="s">
-        <v>19</v>
-      </c>
-      <c r="E12" s="20"/>
-      <c r="F12" s="23"/>
-      <c r="G12" s="23"/>
-    </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="31.5" customFormat="1" s="16">
+        <v>30</v>
+      </c>
+      <c r="E12" s="20" t="s">
+        <v>22</v>
+      </c>
+      <c r="F12" s="23" t="s">
+        <v>14</v>
+      </c>
+      <c r="G12" s="23" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="56.25" customFormat="1" s="16">
       <c r="A13" s="17"/>
       <c r="B13" s="18">
         <v>7</v>
       </c>
       <c r="C13" s="22" t="s">
-        <v>18</v>
+        <v>29</v>
       </c>
       <c r="D13" s="22" t="s">
-        <v>20</v>
-      </c>
-      <c r="E13" s="20"/>
-      <c r="F13" s="23"/>
-      <c r="G13" s="23"/>
+        <v>32</v>
+      </c>
+      <c r="E13" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="F13" s="23" t="s">
+        <v>14</v>
+      </c>
+      <c r="G13" s="23" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="19.5">
       <c r="A14" s="1"/>
@@ -1235,7 +1326,7 @@
     <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="18.75">
       <c r="A34" s="1"/>
       <c r="B34" s="26" t="s">
-        <v>21</v>
+        <v>35</v>
       </c>
       <c r="C34" s="27"/>
       <c r="D34" s="27"/>

</xml_diff>

<commit_message>
Update: Added assignment 3 under README.md. Fix: Replaced mangled names with public accessors.
</commit_message>
<xml_diff>
--- a/tests/A02_pixell_test_plan_investment_account.xlsx
+++ b/tests/A02_pixell_test_plan_investment_account.xlsx
@@ -25,7 +25,7 @@
     <t>Developer:</t>
   </si>
   <si>
-    <t>Sven Beitenger</t>
+    <t/>
   </si>
   <si>
     <t>Class Name:</t>
@@ -482,7 +482,7 @@
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="3" applyBorder="1" fontId="4" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="4" applyBorder="1" fontId="5" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="4" applyBorder="1" fontId="5" applyFont="1" fillId="3" applyFill="1" quotePrefix="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="5" applyBorder="1" fontId="5" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">

</xml_diff>